<commit_message>
Primeira versão do portal de notas
</commit_message>
<xml_diff>
--- a/notas.xlsx
+++ b/notas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniloas.com/projetos/FertilidadeSoloAlegreUFES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B08C8F3-20DA-4849-95EA-6EE3B5FE5C5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3816C1EE-FDB0-D34D-8FF5-A24905722401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="20740" windowHeight="11320" xr2:uid="{BB9E0E1E-73DF-4AB6-A949-07A69840CAF7}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28700" windowHeight="17360" xr2:uid="{BB9E0E1E-73DF-4AB6-A949-07A69840CAF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -1421,7 +1421,7 @@
         <v>13</v>
       </c>
       <c r="F27">
-        <v>0.60000000000000009</v>
+        <v>0.6</v>
       </c>
       <c r="G27" t="s">
         <v>10</v>

</xml_diff>